<commit_message>
Day 7 sheet: winners only, labelled by 7-day ROAS
Hemant's rule, ads with $100+ spend in their first 7 days:
ROAS 2.0+ Breakthrough, 1.8-2.0 Scale winner, 1.4-1.8 Winner,
1.0-1.4 Keep running, under 1.0 Check when it has sales and CTR 2%+,
else killed and left out. Under $100 stays out too.

The sheet drops hook, hold, hypothesis and the verdict dropdown; the team
writes only "why it won" and "next iteration" on winners. The Apps
Script sets the new tab up itself, sorts by ROAS, and takes a lock so two
writes cannot add the same row twice; Donnaa also runs one pull at a time.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Kzesa2s2oMMsdnBk97WudF
</commit_message>
<xml_diff>
--- a/ops/day7/Blissta Creative Day 7 Sheet.xlsx
+++ b/ops/day7/Blissta Creative Day 7 Sheet.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Creatives" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Creatives" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -26,7 +26,6 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <name val="Arial"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
     </font>
@@ -58,43 +57,49 @@
   </cellStyleXfs>
   <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
-  <dxfs count="4">
+  <dxfs count="5">
     <dxf>
       <fill>
         <patternFill patternType="solid">
-          <fgColor rgb="00B7E1CD"/>
-          <bgColor rgb="00B7E1CD"/>
+          <fgColor rgb="0093C47D"/>
+          <bgColor rgb="0093C47D"/>
         </patternFill>
       </fill>
     </dxf>
     <dxf>
       <fill>
         <patternFill patternType="solid">
-          <fgColor rgb="00F4C7C3"/>
-          <bgColor rgb="00F4C7C3"/>
+          <fgColor rgb="00B6D7A8"/>
+          <bgColor rgb="00B6D7A8"/>
         </patternFill>
       </fill>
     </dxf>
     <dxf>
       <fill>
         <patternFill patternType="solid">
-          <fgColor rgb="00D9D9D9"/>
-          <bgColor rgb="00D9D9D9"/>
+          <fgColor rgb="00D9EAD3"/>
+          <bgColor rgb="00D9EAD3"/>
         </patternFill>
       </fill>
     </dxf>
     <dxf>
       <fill>
         <patternFill patternType="solid">
-          <fgColor rgb="00EA9999"/>
-          <bgColor rgb="00EA9999"/>
+          <fgColor rgb="00FFF2CC"/>
+          <bgColor rgb="00FFF2CC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00FCE5CD"/>
+          <bgColor rgb="00FCE5CD"/>
         </patternFill>
       </fill>
     </dxf>
@@ -460,26 +465,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q1"/>
+  <dimension ref="A1:K1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="38" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="20" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="16" customWidth="1" min="6" max="6"/>
-    <col width="14" customWidth="1" min="7" max="7"/>
-    <col width="12" customWidth="1" min="8" max="8"/>
-    <col width="40" customWidth="1" min="9" max="9"/>
-    <col width="12" customWidth="1" min="10" max="10"/>
-    <col width="10" customWidth="1" min="11" max="11"/>
-    <col width="9" customWidth="1" min="12" max="12"/>
-    <col width="9" customWidth="1" min="13" max="13"/>
-    <col width="9" customWidth="1" min="14" max="14"/>
-    <col width="10" customWidth="1" min="15" max="15"/>
-    <col width="11" customWidth="1" min="16" max="16"/>
-    <col width="40" customWidth="1" min="17" max="17"/>
+    <col width="45" customWidth="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="10" max="10"/>
+    <col width="40" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -495,102 +486,68 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Angle</t>
+          <t>Launch date</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Avatar / door</t>
+          <t>Day 7 date</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Format</t>
+          <t>Spend</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Type (Part 5)</t>
+          <t>ROAS</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>Owner</t>
+          <t>CPA</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>Launch date</t>
+          <t>CTR</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>Hypothesis (before launch)</t>
+          <t>Label</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>Day 7 date</t>
+          <t>Why it won</t>
         </is>
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
-          <t>Spend</t>
-        </is>
-      </c>
-      <c r="L1" s="1" t="inlineStr">
-        <is>
-          <t>Hook %</t>
-        </is>
-      </c>
-      <c r="M1" s="1" t="inlineStr">
-        <is>
-          <t>Hold</t>
-        </is>
-      </c>
-      <c r="N1" s="1" t="inlineStr">
-        <is>
-          <t>CTR</t>
-        </is>
-      </c>
-      <c r="O1" s="1" t="inlineStr">
-        <is>
-          <t>CPA</t>
-        </is>
-      </c>
-      <c r="P1" s="1" t="inlineStr">
-        <is>
-          <t>Verdict</t>
-        </is>
-      </c>
-      <c r="Q1" s="1" t="inlineStr">
-        <is>
-          <t>Why (one line)</t>
+          <t>Next iteration</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="P2:P5000">
-    <cfRule type="expression" priority="1" dxfId="0">
-      <formula>$P2="winner"</formula>
+  <conditionalFormatting sqref="A2:I5000">
+    <cfRule type="expression" priority="1" dxfId="0" stopIfTrue="1">
+      <formula>ISNUMBER(SEARCH("Breakthrough",$I2))</formula>
     </cfRule>
-    <cfRule type="expression" priority="2" dxfId="1">
-      <formula>$P2="kill"</formula>
+    <cfRule type="expression" priority="2" dxfId="1" stopIfTrue="1">
+      <formula>ISNUMBER(SEARCH("Scale winner",$I2))</formula>
     </cfRule>
-    <cfRule type="expression" priority="3" dxfId="2">
-      <formula>$P2="no read"</formula>
+    <cfRule type="expression" priority="3" dxfId="2" stopIfTrue="1">
+      <formula>ISNUMBER(SEARCH("Winner",$I2))</formula>
+    </cfRule>
+    <cfRule type="expression" priority="4" dxfId="3" stopIfTrue="1">
+      <formula>ISNUMBER(SEARCH("Keep running",$I2))</formula>
+    </cfRule>
+    <cfRule type="expression" priority="5" dxfId="4" stopIfTrue="1">
+      <formula>ISNUMBER(SEARCH("Check",$I2))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I2:I5000">
-    <cfRule type="expression" priority="4" dxfId="3">
-      <formula>AND($H2&lt;&gt;"",LEN(TRIM($I2))=0)</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <dataValidations count="1">
-    <dataValidation sqref="P2:P5000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Verdict" error="Pick winner, iterate, fix, kill or no read." type="list">
-      <formula1>"winner,iterate,fix,kill,no read"</formula1>
-    </dataValidation>
-  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Day 7 sheet: Killed tab, ad preview links, Testing column
Winners tab keeps the ROAS labels; ads with $100+ spend and no label go to
a Killed tab so the angles that died are on record. Every row gets a link
to the ad (Meta preview link, else Ads Manager) and a Testing column for
the hypothesis; Killed rows get "What we learned". Dates are written as
yyyy-mm-dd text so the sheet shows the launch day Donnaa sent instead of
shifting it by the sheet's time zone.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Kzesa2s2oMMsdnBk97WudF
</commit_message>
<xml_diff>
--- a/ops/day7/Blissta Creative Day 7 Sheet.xlsx
+++ b/ops/day7/Blissta Creative Day 7 Sheet.xlsx
@@ -7,7 +7,8 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Creatives" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Winners" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Killed" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -62,48 +63,6 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
-  <dxfs count="5">
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="0093C47D"/>
-          <bgColor rgb="0093C47D"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="00B6D7A8"/>
-          <bgColor rgb="00B6D7A8"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="00D9EAD3"/>
-          <bgColor rgb="00D9EAD3"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="00FFF2CC"/>
-          <bgColor rgb="00FFF2CC"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="00FCE5CD"/>
-          <bgColor rgb="00FCE5CD"/>
-        </patternFill>
-      </fill>
-    </dxf>
-  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <indexedColors>
@@ -465,13 +424,8 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K1"/>
+  <dimension ref="A1:M1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="45" customWidth="1" min="1" max="1"/>
-    <col width="40" customWidth="1" min="10" max="10"/>
-    <col width="40" customWidth="1" min="11" max="11"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
@@ -481,73 +435,142 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
+          <t>Ad</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
           <t>Product</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Launch date</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Day 7 date</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Spend</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>ROAS</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>CPA</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>CTR</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Label</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Testing</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>Why it won</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>Next iteration</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="A2:I5000">
-    <cfRule type="expression" priority="1" dxfId="0" stopIfTrue="1">
-      <formula>ISNUMBER(SEARCH("Breakthrough",$I2))</formula>
-    </cfRule>
-    <cfRule type="expression" priority="2" dxfId="1" stopIfTrue="1">
-      <formula>ISNUMBER(SEARCH("Scale winner",$I2))</formula>
-    </cfRule>
-    <cfRule type="expression" priority="3" dxfId="2" stopIfTrue="1">
-      <formula>ISNUMBER(SEARCH("Winner",$I2))</formula>
-    </cfRule>
-    <cfRule type="expression" priority="4" dxfId="3" stopIfTrue="1">
-      <formula>ISNUMBER(SEARCH("Keep running",$I2))</formula>
-    </cfRule>
-    <cfRule type="expression" priority="5" dxfId="4" stopIfTrue="1">
-      <formula>ISNUMBER(SEARCH("Check",$I2))</formula>
-    </cfRule>
-  </conditionalFormatting>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:L1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Creative</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Ad</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Product</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Launch date</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Day 7 date</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Spend</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>ROAS</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>CPA</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>CTR</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Label</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Testing</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>What we learned</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>